<commit_message>
feat: add manual one-click update, integrate sync converter, and update data
</commit_message>
<xml_diff>
--- a/水果市場評論貼文_匯入進度.xlsx
+++ b/水果市場評論貼文_匯入進度.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="2"/>
@@ -3708,6 +3708,165 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>如果農夫玩皮克敏會怎麼樣？</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>如果農夫玩皮克敏會怎麼樣？</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>如果農夫玩皮克敏會怎麼樣？
+好多人再玩，已經筆記起來，感謝大家提供方法🙏🙏
+新手第一天😆
+會喔+防水袋
+防水袋必備👍
+筆記🖊️🖋️，謝謝
+好喔😄
+擔心手機過熱
+看來是過來人🖋️🖊️
+筆記🖊️🖋️，謝謝
+擔心
+筆記🖊️🖋️，謝謝
+筆記🖊️🖋️，謝謝
+今天是新手😆
+蛤.....
+筆記🖊️🖋️，謝謝
+蛤？</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>每週評青菜市場 7/20-7/26</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>🔊每週評青菜市場 7/20-7/26
+ ⚠️這週參考價值較低（因颱風對產區的不確定性），以下預測僅供參考：
+🎈蔬菜漲價建議觀望：
+超級貴：香菜
+很貴：玉米筍-帶殼（北部高雄）、奶油白菜（中南部）、水耕萵苣、芥藍芽（量少）、三星蔥（僅北部）
+貴：牛番茄（僅北部）、南瓜（阿成.圓形）、龍鬚菜、高麗菜-初秋、包心白菜（僅高雄）、小白菜、奶油白菜（北部屏東）、青江菜（北部）、A菜、福山萵苣-大陸妹、油菜（北南部）、粉蔥、韭菜（北部）
+微漲：秋葵（北部）、小黃瓜（北部屏東）、牛番茄（中南部）、彩椒（北部高雄）、青椒、菜豆、敏豆、櫛瓜（北部高雄）、包心白菜、青江菜（中南部）、皇宮菜（北部）、空心菜（北南部）、水空心菜（僅北部）、福山萵苣-大陸妹（僅台中）、小芥菜、莧菜、油菜（中部）、地瓜葉（北部高雄）、紅鳳菜、水蓮、玉米筍-帶殼（中南部）、糯米玉米（僅高雄）、玉米-白龍王（量少）、芹菜、韭菜（中南部）、綠竹筍（僅北部）、粉蔥（僅台中）
+🟨蔬菜價格持平不貴：秋葵（中部）、大黃瓜、小黃瓜（中南部）、冬瓜、絲瓜、白苦瓜、珍珠苦瓜、蒲瓜、茄子、彩椒（中南部）、櫛瓜（中南部）、高麗菜-硬種、小白菜（僅屏東）、皇宮菜（中南部）、空心菜（中部）、水空心菜（僅台中）、地瓜葉（中南部）、糯米玉米、黃玉米、紅蘿蔔、麻竹筍、竹筍-烏殼綠、蓮藕（北部高雄）、地瓜57號（南部）、地瓜66號（僅高雄）、粉蔥（僅屏東）、洋蔥
+🟩地板價：秋葵（南部）、蒲瓜（僅台中屏東）、牛番茄（僅豐原）、彩椒（僅台中屏東）、敏豆（僅台中）、糯米玉米（僅台中屏東）、包心白菜（僅台中）、地瓜葉（僅屏東）、麻竹筍（僅台中）、馬鈴薯、豆薯、地瓜57號（北中部）、地瓜66號、芋頭、蓮藕（中南部）、糯米椒、芹菜（僅屏東）、九層塔
+註1：雜糧豆類、菇類、豆芽菜不列入參考。
+註2：初秋高麗菜產量減少價格微降、改良種高麗菜產量增加價格降多；大白菜產能減少，價格持平
+註3：（北農）因逢明日休市，預期需求增加，由於到貨量持續增加，承銷人購買意願趨緩，買氣尚可，交易市況平順，各菜種行情價格漲跌互見。
+註4：小編自己意見：
+1.葉菜區產量減少價格漲，產量未恢復正常產量，颱風後價格維持中高水位
+2.瓜果類產量增加，價格持平
+3.玉米筍-帶殼、紅辣椒、朝天椒產量大減，價格穩定漲價，猜測有災情
+4.開始進口中國木瓜型南瓜/替代國內本產阿成南瓜，價格繼續觀察
+氣象報告：多日午後雷陣雨導致蔬菜產區照顧難度增加，繼續觀察高麗菜-初秋及整體綠色葉菜類產量；
+下週開始午後中部以北、宜花地區與各山區將普遍出現雷陣雨。目前菲律賓東方海面至關島一帶的熱帶擾動已出現發展跡象</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>🔊每週評青菜市場 7/20-7/26
+ ⚠️這週參考價值較低（因颱風對產區的不確定性），以下預測僅供參考：
+🎈蔬菜漲價建議觀望：
+超級貴：香菜
+很貴：玉米筍-帶殼（北部高雄）、奶油白菜（中南部）、水耕萵苣、芥藍芽（量少）、三星蔥（僅北部）
+貴：牛番茄（僅北部）、南瓜（阿成.圓形）、龍鬚菜、高麗菜-初秋、包心白菜（僅高雄）、小白菜、奶油白菜（北部屏東）、青江菜（北部）、A菜、福山萵苣-大陸妹、油菜（北南部）、粉蔥、韭菜（北部）
+微漲：秋葵（北部）、小黃瓜（北部屏東）、牛番茄（中南部）、彩椒（北部高雄）、青椒、菜豆、敏豆、櫛瓜（北部高雄）、包心白菜、青江菜（中南部）、皇宮菜（北部）、空心菜（北南部）、水空心菜（僅北部）、福山萵苣-大陸妹（僅台中）、小芥菜、莧菜、油菜（中部）、地瓜葉（北部高雄）、紅鳳菜、水蓮、玉米筍-帶殼（中南部）、糯米玉米（僅高雄）、玉米-白龍王（量少）、芹菜、韭菜（中南部）、綠竹筍（僅北部）、粉蔥（僅台中）
+🟨蔬菜價格持平不貴：秋葵（中部）、大黃瓜、小黃瓜（中南部）、冬瓜、絲瓜、白苦瓜、珍珠苦瓜、蒲瓜、茄子、彩椒（中南部）、櫛瓜（中南部）、高麗菜-硬種、小白菜（僅屏東）、皇宮菜（中南部）、空心菜（中部）、水空心菜（僅台中）、地瓜葉（中南部）、糯米玉米、黃玉米、紅蘿蔔、麻竹筍、竹筍-烏殼綠、蓮藕（北部高雄）、地瓜57號（南部）、地瓜66號（僅高雄）、粉蔥（僅屏東）、洋蔥
+🟩地板價：秋葵（南部）、蒲瓜（僅台中屏東）、牛番茄（僅豐原）、彩椒（僅台中屏東）、敏豆（僅台中）、糯米玉米（僅台中屏東）、包心白菜（僅台中）、地瓜葉（僅屏東）、麻竹筍（僅台中）、馬鈴薯、豆薯、地瓜57號（北中部）、地瓜66號、芋頭、蓮藕（中南部）、糯米椒、芹菜（僅屏東）、九層塔
+註1：雜糧豆類、菇類、豆芽菜不列入參考。
+註2：初秋高麗菜產量減少價格微降、改良種高麗菜產量增加價格降多；大白菜產能減少，價格持平
+註3：（北農）因逢明日休市，預期需求增加，由於到貨量持續增加，承銷人購買意願趨緩，買氣尚可，交易市況平順，各菜種行情價格漲跌互見。
+註4：小編自己意見：
+1.葉菜區產量減少價格漲，產量未恢復正常產量，颱風後價格維持中高水位
+2.瓜果類產量增加，價格持平
+3.玉米筍-帶殼、紅辣椒、朝天椒產量大減，價格穩定漲價，猜測有災情
+4.開始進口中國木瓜型南瓜/替代國內本產阿成南瓜，價格繼續觀察
+氣象報告：多日午後雷陣雨導致蔬菜產區照顧難度增加，繼續觀察高麗菜-初秋及整體綠色葉菜類產量；
+下週開始午後中部以北、宜花地區與各山區將普遍出現雷陣雨。目前菲律賓東方海面至關島一帶的熱帶擾動已出現發展跡象
+高麗菜-初秋拍賣量明顯減少
+綠色葉菜類北中部產量減少，繼續觀察
+其實有點難過
+蛛絲馬跡，陸續有些進口消息，不跑拍賣市跑行口居多
+💪🙏</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>很誇張</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="n">
+        <v>46222</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>很誇張
+梧棲大排兩側的頂寮里與下寮里低窪農地遭遇海水倒灌後其實很嚴重😭
+像是人體敗血症那般會引發系統性的連鎖崩潰， 人體的敗血症，是細菌和毒素隨著血液流到全身，引發器官衰竭；而海水倒灌，則是高濃度的鹽水隨著水流滲透進整片土地的毛細孔，讓整片農田作物急性中毒死亡
+海水的鹹度太高，嚴重的「高滲透壓」把活生生的植物細胞泡進濃鹽水裡，作物的根部不但吸不到水，體內的水分反而會被整隻吸出來，短短幾天內，作物就會因為這種急性脫水而集體枯死
+再來，土壤窒息跟有益菌會死光：海水中的鈉離子會破壞泥土的結構，讓原本鬆軟、有空氣的土壤崩塌，緊密黏成一塊，直接切斷土壤的空氣，讓植物根部像溺水一樣窒息變黑，同時，土裡原本幫忙維持地力的好菌，也會因為太鹹而集體陣亡，讓土地徹底失去免疫力
+最後會留下嚴重後遺症，海水退了不代表沒事，大量的鹽分已經死死卡在泥土深處，只要出太陽、水分蒸發，這些鹽分就會順著泥土微管再度被抽回地表，讓土地長期硬化、無法耕作。 這不是普通的淹水，土地已經受到難以挽回的傷害</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>很誇張
+梧棲大排兩側的頂寮里與下寮里低窪農地遭遇海水倒灌後其實很嚴重😭
+像是人體敗血症那般會引發系統性的連鎖崩潰， 人體的敗血症，是細菌和毒素隨著血液流到全身，引發器官衰竭；而海水倒灌，則是高濃度的鹽水隨著水流滲透進整片土地的毛細孔，讓整片農田作物急性中毒死亡
+海水的鹹度太高，嚴重的「高滲透壓」把活生生的植物細胞泡進濃鹽水裡，作物的根部不但吸不到水，體內的水分反而會被整隻吸出來，短短幾天內，作物就會因為這種急性脫水而集體枯死
+再來，土壤窒息跟有益菌會死光：海水中的鈉離子會破壞泥土的結構，讓原本鬆軟、有空氣的土壤崩塌，緊密黏成一塊，直接切斷土壤的空氣，讓植物根部像溺水一樣窒息變黑，同時，土裡原本幫忙維持地力的好菌，也會因為太鹹而集體陣亡，讓土地徹底失去免疫力
+最後會留下嚴重後遺症，海水退了不代表沒事，大量的鹽分已經死死卡在泥土深處，只要出太陽、水分蒸發，這些鹽分就會順著泥土微管再度被抽回地表，讓土地長期硬化、無法耕作。 這不是普通的淹水，土地已經受到難以挽回的傷害
+誰開的？梧棲大排閘門「離奇開啟」海水倒灌 農民崩潰：二期稻作毀了
+https://tw.news.yahoo.com/share/b46d9812-ce06-3bbc-bb7e-ed332b42d1e2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" display="https://www.threads.com/@abc89151207" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: change fruit market browse page to show bulleted raw JSON list based on Thunderbit template
</commit_message>
<xml_diff>
--- a/水果市場評論貼文_匯入進度.xlsx
+++ b/水果市場評論貼文_匯入進度.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="2"/>
@@ -3867,6 +3867,365 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>46225</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......
+但是一想到這隻狗，今天還沒有被好好的揉揉揉、捏捏捏，身心健康可能會受影響
+為了牠好，我又心軟了，手邊的事先放著，我先來履行我身為按摩師傅（摸胸肌？）的職責</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......
+但是一想到這隻狗，今天還沒有被好好的揉揉揉、捏捏捏，身心健康可能會受影響
+為了牠好，我又心軟了，手邊的事先放著，我先來履行我身為按摩師傅（摸胸肌？）的職責
+我是不會承認因為接下來接受委託種9分地的豆子想昏倒躺平-------&gt;假的
+科學研究指出，狗的一生只有我們大約七分之一的時間，牠的五分鐘等於我的半小時，一想到牠用珍貴的青春在等我，我又心軟了--------------&gt;真的</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="n">
+        <v>46225</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......
+但是一想到這隻狗，今天還沒有被好好的揉揉揉、捏捏捏，身心健康可能會受影響
+為了牠好，我又心軟了，手邊的事先放著，我先來履行我身為按摩師傅（摸胸肌？）的職責</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>我本來打算繼續認真工作做事的......
+但是一想到這隻狗，今天還沒有被好好的揉揉揉、捏捏捏，身心健康可能會受影響
+為了牠好，我又心軟了，手邊的事先放著，我先來履行我身為按摩師傅（摸胸肌？）的職責
+我是不會承認因為接下來接受委託種9分地的豆子想昏倒躺平-------&gt;假的
+科學研究指出，狗的一生只有我們大約七分之一的時間，牠的五分鐘等於我的半小時，一想到牠用珍貴的青春在等我，我又心軟了--------------&gt;真的</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+對的，生鮮季節在這時候</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+這個月台產青花菜幾乎沒有，能存活的高山區能種，但因為進口競爭的關係，青花菜不是好項目，大部分種高麗菜、大白菜、櫛瓜、敏豆等等其他更好賣</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+一定是</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+好氣！</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+這個月台產青花菜幾乎沒有，能存活的高山區能種，但因為進口競爭的關係，青花菜不是好項目，大部分種高麗菜、大白菜、櫛瓜、敏豆等等其他更好賣</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+讚讚！</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>abc89151207</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>農民日常</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>拜託了，農產詐騙又開始死灰復燃
+有在追我的蔬果週報一定會知道的事❗❗❗
+1.青花菜（青花椰菜）現在99%以上都是進口的，不可能每天新鮮採
+2.愛文芒果現在不可能太便宜，價格漲而且還搶手，產季尾聲已經快要沒有了
+3.初秋高麗菜一顆30塊怎麼可能？？
+是不是當令蔬菜產期、產量減少價格有沒有漲、有沒有天災？週報裡都有寫原因
+是的！高山高麗菜，最近價格較高 ..</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" display="https://www.threads.com/@abc89151207" r:id="rId1"/>

</xml_diff>